<commit_message>
chore: update excel data
</commit_message>
<xml_diff>
--- a/data/evidence/data_procesor/qualityReportIDBTest_May_2026.xlsx
+++ b/data/evidence/data_procesor/qualityReportIDBTest_May_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LGSM065\Music\Quality_Report_IDB\data\evidence\data_procesor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE9A81B9-3848-4FC5-A6C0-E6821EFEAE66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC6681B2-C73F-4B3C-9AD6-E81FC12A6BA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="17500" activeTab="1" xr2:uid="{1BFDC0BB-3264-4789-A41B-B16DE7BD9ED5}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="17500" activeTab="2" xr2:uid="{1BFDC0BB-3264-4789-A41B-B16DE7BD9ED5}"/>
   </bookViews>
   <sheets>
     <sheet name="SI" sheetId="13" r:id="rId1"/>
@@ -559,32 +559,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">otal workload </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>97 (79% completed)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> indicates delay risk. No defects reported so far; need to review workload completion drivers and ensure no gaps in defect identification during ongoing execution.</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">Total workload </t>
     </r>
     <r>
@@ -753,6 +727,32 @@
   </si>
   <si>
     <t>2 task still in code review, 4 task in progress</t>
+  </si>
+  <si>
+    <r>
+      <t>Total workload 97</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (80% completed)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> indicates delay risk. No defects reported so far; need to review workload completion drivers and ensure no gaps in defect identification during ongoing execution.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -3436,7 +3436,7 @@
         <v>97</v>
       </c>
       <c r="K3" s="99">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="L3" s="99">
         <v>0</v>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="N3" s="100">
         <f t="shared" si="0"/>
-        <v>0.79381443298969068</v>
+        <v>0.80412371134020622</v>
       </c>
       <c r="O3" s="102">
         <f t="shared" si="0"/>
@@ -3457,7 +3457,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="Q3" s="133" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:17" ht="43.25" customHeight="1">
@@ -3496,7 +3496,7 @@
         <v>1</v>
       </c>
       <c r="Q4" s="133" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5" spans="1:17" ht="43.25" customHeight="1">
@@ -3535,7 +3535,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="Q5" s="133" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="6" spans="1:17" ht="43.25" customHeight="1">
@@ -3574,7 +3574,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="Q6" s="133" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="43.25" customHeight="1">
@@ -3613,7 +3613,7 @@
         <v>1</v>
       </c>
       <c r="Q7" s="133" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="8" spans="1:17" ht="43.25" customHeight="1">
@@ -3652,7 +3652,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="Q8" s="133" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="9" spans="1:17" ht="43.25" customHeight="1">
@@ -3691,7 +3691,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="Q9" s="133" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="10" spans="1:17">
@@ -5073,7 +5073,7 @@
         <v>1</v>
       </c>
       <c r="Q7" s="133" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="U7" s="122">
         <v>48</v>
@@ -5453,10 +5453,10 @@
     <row r="3" spans="1:44" ht="43.25" customHeight="1">
       <c r="B3" s="96"/>
       <c r="C3" s="135" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D3" s="135" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E3" s="97"/>
       <c r="F3" s="97"/>
@@ -6397,7 +6397,7 @@
     <row r="3" spans="1:29" ht="43.25" customHeight="1">
       <c r="B3" s="96"/>
       <c r="C3" s="135" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D3" s="96"/>
       <c r="E3" s="97"/>
@@ -6557,7 +6557,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="Q5" s="133" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="U5" s="134">
         <v>15</v>
@@ -6620,7 +6620,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="Q6" s="133" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="U6" s="134">
         <v>6</v>
@@ -6809,7 +6809,7 @@
         <v>1</v>
       </c>
       <c r="Q9" s="133" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="U9" s="122">
         <v>25</v>
@@ -7122,6 +7122,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="0e42490b-809c-485c-a127-0ea0c2e12b0b" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="65d4c795-5362-4472-a968-0591b4901adb">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101004DC2141999F3A34989E45D589C11CC4C" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fffa584a95f0f180d3ff00a1c6b20f2c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="65d4c795-5362-4472-a968-0591b4901adb" xmlns:ns3="0e42490b-809c-485c-a127-0ea0c2e12b0b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6b1bfd8c2e9b957913a6f07f22fa0e9e" ns2:_="" ns3:_="">
     <xsd:import namespace="65d4c795-5362-4472-a968-0591b4901adb"/>
@@ -7316,17 +7327,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="0e42490b-809c-485c-a127-0ea0c2e12b0b" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="65d4c795-5362-4472-a968-0591b4901adb">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E1A5E9D6-D263-445D-A876-96A4702D14D9}">
   <ds:schemaRefs>
@@ -7336,6 +7336,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EEBA5460-617B-4FEF-BA90-2B9D69F7B2B2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="0e42490b-809c-485c-a127-0ea0c2e12b0b"/>
+    <ds:schemaRef ds:uri="65d4c795-5362-4472-a968-0591b4901adb"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1BCBA3EB-3C5C-4F4D-BA3B-BDBA6C49B7D0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7354,17 +7365,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EEBA5460-617B-4FEF-BA90-2B9D69F7B2B2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="0e42490b-809c-485c-a127-0ea0c2e12b0b"/>
-    <ds:schemaRef ds:uri="65d4c795-5362-4472-a968-0591b4901adb"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{29b7d34e-545d-48ef-aae6-8370e78eb279}" enabled="1" method="Privileged" siteId="{fab2d60f-e614-4f9d-b2ad-9fb1397f2efe}" removed="0"/>

</xml_diff>

<commit_message>
chore: update excel data file again
</commit_message>
<xml_diff>
--- a/data/evidence/data_procesor/qualityReportIDBTest_May_2026.xlsx
+++ b/data/evidence/data_procesor/qualityReportIDBTest_May_2026.xlsx
@@ -7122,17 +7122,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="0e42490b-809c-485c-a127-0ea0c2e12b0b" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="65d4c795-5362-4472-a968-0591b4901adb">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101004DC2141999F3A34989E45D589C11CC4C" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fffa584a95f0f180d3ff00a1c6b20f2c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="65d4c795-5362-4472-a968-0591b4901adb" xmlns:ns3="0e42490b-809c-485c-a127-0ea0c2e12b0b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6b1bfd8c2e9b957913a6f07f22fa0e9e" ns2:_="" ns3:_="">
     <xsd:import namespace="65d4c795-5362-4472-a968-0591b4901adb"/>
@@ -7327,6 +7316,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="0e42490b-809c-485c-a127-0ea0c2e12b0b" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="65d4c795-5362-4472-a968-0591b4901adb">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E1A5E9D6-D263-445D-A876-96A4702D14D9}">
   <ds:schemaRefs>
@@ -7336,17 +7336,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EEBA5460-617B-4FEF-BA90-2B9D69F7B2B2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="0e42490b-809c-485c-a127-0ea0c2e12b0b"/>
-    <ds:schemaRef ds:uri="65d4c795-5362-4472-a968-0591b4901adb"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1BCBA3EB-3C5C-4F4D-BA3B-BDBA6C49B7D0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7365,6 +7354,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EEBA5460-617B-4FEF-BA90-2B9D69F7B2B2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="0e42490b-809c-485c-a127-0ea0c2e12b0b"/>
+    <ds:schemaRef ds:uri="65d4c795-5362-4472-a968-0591b4901adb"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{29b7d34e-545d-48ef-aae6-8370e78eb279}" enabled="1" method="Privileged" siteId="{fab2d60f-e614-4f9d-b2ad-9fb1397f2efe}" removed="0"/>

</xml_diff>